<commit_message>
docs: refactor access documentation for unrestricted users and add supporting data templates
</commit_message>
<xml_diff>
--- a/data/lideres_projeto.xlsx
+++ b/data/lideres_projeto.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -680,18 +680,6 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Superintendência</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>GIZ_2025_01, ARTERY PRODUCOES_2025_01, CERAS JOHNSON_PES_2025_01, SWAROVSKI_2025_01, FUNDAÇÃO BANCO DO BRASIL_2026_01, DELL 2022_1, DELL 2024_1, DELL 2025_01, FUMCAD BERURI, FUMCAD EIRUNEPÉ II, FUMCAD ITAPIRANGA II - FINALIZADO, FUMCAD MANICORÉ, FUMCAD MARAÃ IV, FUMCAD TEFÉ II, FUNDO AMAZONIA_PIRÃO_2026_01, Pelo Rio Expedições Educativas Turismo Ltda. PEL_2024_1, BRAZIL FOUNDATION_CONSULTORIA_2025_01, RENAISSANCE HOTELARIA_2026_01, FUNDAÇÃO AVINA_2025_01, RECOFARMA INDUSTRIA DO AM_2024_01, Associação Vale - Campanha Seca Amazonica 2023, ALUGUEL ESPAÇO FAS_2025_01, ALUGUEL ESPAÇO FAS_2026_01, BENFEITORIA_2024_01, DOAÇÃO AVULSA DE PF_2025_01, DOAÇÃO AVULSA DE PF_2026_01, MITSUBISHI MIT_2025_02, WELIGTH_2026_01, Rendimentos_RECOFARMA INDUSTRIA DO AM_2024_01, WINLOGIS GESTAO LOGISTICA_2025_01, XPRIZE_2024_01, Youth Climate Leaders_2024_1, Youth Climate Leaders_2025_01, BRADESCO_2025_01, ABDI_2025_01, AMAZONIA ANDES 2025_01, Amazônia Andes AAF2024_1, Amazônia Andes II AAF2020_1, BANZEIRO DA ESPERANÇA - COP 30, BASF_2024_1, Instituto Clima e Sociedade_ICS_2025_01, INSTITUTO VIRADA SUSTENTÁVEL_2025_COP30, MITSUBISHI_2025_01, NORTE ENERGIA S.A_2022_1, REM MT - FUNBIO 2023, FUNDO AMAZONIA_PROSPERA_2026_01, Associação Brazil Foundation_2023_2, MITSUBISHI MIT_2024_1, CERAS JOHNSON_PSF_2025_01, IDIS_UMANE_2025_02, IDIS_VALE_2025_01, Ilana Benchimol Minev IBM 2025_01, INSTITUTO GPA_2025_01, Nota de Débito 01/2026 - IDIS, KfW-SBIO, KfW 2023_01_Floresta em Pé_Amazonas, KfW 2023_01_Floresta em Pé_AT, KfW 2023_01_Floresta em Pé_Gestão ACCF, KfW 2023_01_Floresta em Pé_Pará, KFW 2024_01 - REM MT Pré Operacional, KFW 2024_01_SOCIOBIO_Pré Operacional_MMA, KFW_2024_02_REM MT, KFW_2024_02_REM MT_Gestão, KFW_2024_03_REM MT, KFW_2024_03_REM MT_GESTÃO_ACCF, KFW_2025_01_REM MT, KFW_2025_01_REM MT_Gestão, KFW_2026_01_SOCIOBIOECONOMIA, LUCIANO ARBEX SARKIS_2025_01, TRANSALEX CARGAS_2024_01, AMAZONIANDO_2025_01, Associação Vero 2024_1, CANDIDO BOTELHO BRACHER 2025, CANDIDO BOTELHO BRACHER 2026, Carrefour_2024_1, CONSULADO DA MULHER_2025_01, MARRIOT 2024_01, Adiantamento de despesas 03/2026 - PPI ATL 2026, BRAZIL FOUNDATION_2024_01, CONFEDERAÇÃO BRASILEIRA DE CANOAGEM_2024_01, Denis Benchimol Minev DBM 2024_01, Ilana Benchimol Minev IBM 2024_1, PF_Pessoa Fisica_2024_Centro de Treinamento Indígena de Arco e Flecha, STRIPE BRASIL SOLUCOES - Plataforma de captação 2023, STRIPE BRASIL_2026_01, THE WALL_Globo Comunicações, UK ONLINE GIVING UK 2022_01, UK ONLINE GIVING 2025_01, BNDES_2024_1, Movimento Bem Maior MBM_2022_01, Associação Vale para o desenvolvimento sustentável_2023_1, BASF_2024_2, GEAPP_2025_01, AMAZONAS SHOPPING_2025_01, Denis Minev_2023_01, FUNDAÇÃO DOM CABRAL_2025_01, Fundo L'Oréal_2024_1, INSTITUTO DE CONSERVAÇÃO E DESENVOLVIMENTO SUSTENTÁVEL DA AMAZÔNIA - IDESAM - 2024_1, Louis Vuitton LVMH_2023_1, Rendimentos_Louis Vuitton LVMH_2023_1, SAP 2024_01, Taxa administrativa_INSTITUTO DE CONSERVAÇÃO E DESENVOLVIMENTO SUSTENTÁVEL DA AMAZÔNIA - IDESAM - 2024_1, Louis Vuitton LVMH_2023_1_Rendimentos, MACKENZIE_RH_2025_2, REM MT FUNBIO 2023, LUCI FERREIRO LONGUI_2026_01, MACKENZIE_2025_1, MACKENZIE_2025_2, PAR - Fundo Amazônia, YOUTH CLIMATE_2026_01</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>